<commit_message>
vault backup: 2026-03-09 20:53:38
</commit_message>
<xml_diff>
--- a/员工自评表-李世龙.xlsx
+++ b/员工自评表-李世龙.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\任职评审\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91C7BF2E-9266-43F8-916B-B9B1D7B9EBA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D71AA2EC-2406-4B80-AA27-98ED51D35B80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,9 +72,6 @@
     <t>您认为自己今后需要改进和完善的部分</t>
   </si>
   <si>
-    <t>其他：</t>
-  </si>
-  <si>
     <t>姓名：李世龙</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -83,7 +80,11 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>所在部门：研发部三部一组</t>
+    <t>其他：</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>所在部门：研发部三部</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -571,13 +572,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -664,7 +665,7 @@
     </row>
     <row r="12" spans="1:3" ht="84" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="10" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>

</xml_diff>

<commit_message>
vault backup: 2026-03-10 17:23:06
</commit_message>
<xml_diff>
--- a/员工自评表-李世龙.xlsx
+++ b/员工自评表-李世龙.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D71AA2EC-2406-4B80-AA27-98ED51D35B80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F93644-32C4-40EF-A5EA-3863812497F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>类别</t>
   </si>
@@ -85,6 +85,10 @@
   </si>
   <si>
     <t>所在部门：研发部三部</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>负责BES AppServer标准版、企业版、LITE版、SpringBoot版的需求开发及BUG修复</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -599,7 +603,9 @@
       <c r="B3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="8"/>
+      <c r="C3" s="8" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A4" s="13"/>

</xml_diff>

<commit_message>
vault backup: 2026-03-23 02:08:40
</commit_message>
<xml_diff>
--- a/员工自评表-李世龙.xlsx
+++ b/员工自评表-李世龙.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Data\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F93644-32C4-40EF-A5EA-3863812497F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867ABFAD-BA01-4808-9895-087EBFEBBD88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8380" yWindow="3510" windowWidth="23910" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>类别</t>
   </si>
@@ -88,7 +88,41 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>负责BES AppServer标准版、企业版、LITE版、SpringBoot版的需求开发及BUG修复</t>
+    <t>1、加深产品宏观理解
+2、保持严谨、注意细节
+3、加强沟通能力，充分理解需求或问题</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>负责AppServer标准版、企业版、LITE版、SpringBoot版及其子组件的需求开发及BUG修复</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>对于新产品或模块，有深入研究的热情。并且上手速度还可以。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>对于中间件产品的开发有些微的不熟悉，之前都是做业务开发，需要对一些中间件的广度和深度都要加强。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>能够和前端、测试、产品等有充分的沟通。基本可以完整的理解其问题</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>对于应用服务器各个模块或子模块都有一定的了解，相关的Bug或需求都有过处理，包括CLI、控制台、Appguard、应用部署等。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>对于Linux操作、熟悉了以前没有接触过的技术栈，如jmeter、jenkins等。源码阅读能力进一步提升，相关技术栈深度进一步加深。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>对于应用服务器的相关模块还需要继续的深入了解。以及相关工具的使用也需要更加熟练。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>对于当前工作技能基本都能熟悉，包括jira、Jenkins、jmeter、以及相关开发技术。如：Java基础知识、数据库、spring框架等。</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -567,14 +601,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.125" customWidth="1"/>
-    <col min="2" max="2" width="32.5" customWidth="1"/>
-    <col min="3" max="3" width="74" customWidth="1"/>
+    <col min="1" max="1" width="23.08984375" customWidth="1"/>
+    <col min="2" max="2" width="32.453125" customWidth="1"/>
+    <col min="3" max="3" width="78.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -585,7 +619,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -596,7 +630,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:3" ht="28" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>3</v>
       </c>
@@ -604,72 +638,88 @@
         <v>4</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.15">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="13"/>
       <c r="B4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="8"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="C4" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="28" x14ac:dyDescent="0.25">
       <c r="A5" s="14"/>
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="8"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="C5" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="8"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="C6" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="28" x14ac:dyDescent="0.25">
       <c r="A7" s="13"/>
       <c r="B7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="8"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="C7" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="28" x14ac:dyDescent="0.25">
       <c r="A8" s="13"/>
       <c r="B8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="8"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="C8" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="14"/>
       <c r="B9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="9"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="C9" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="28" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="8"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="C10" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="42" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="8"/>
-    </row>
-    <row r="12" spans="1:3" ht="84" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C11" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="84" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>18</v>
       </c>
@@ -691,7 +741,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -702,7 +752,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>